<commit_message>
always allow "NULL" in date columns
</commit_message>
<xml_diff>
--- a/tests/data/test_shift_ignore/workbook.xlsx
+++ b/tests/data/test_shift_ignore/workbook.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/shift_ignore/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/test_shift_ignore/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF62A11-882D-6C40-8A51-0F539D53902D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3317E5C-EF85-7D40-A1E7-79D10FFD20ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="3480" windowWidth="28800" windowHeight="15600" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="page-desc" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>foo</t>
   </si>
@@ -139,6 +138,18 @@
   </si>
   <si>
     <t>this one has spaces</t>
+  </si>
+  <si>
+    <t>nuh56</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>oo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nuh57 </t>
   </si>
 </sst>
 </file>
@@ -602,7 +613,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640D4E5C-A101-794A-8A66-BA19A027AC5F}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="50.6640625" customWidth="1"/>
@@ -698,6 +709,25 @@
         <v>32</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>